<commit_message>
upload to lab github
</commit_message>
<xml_diff>
--- a/data/ref_affinity.xlsx
+++ b/data/ref_affinity.xlsx
@@ -20,7 +20,19 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="27">
+  <si>
+    <t xml:space="preserve">PBD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">peptide</t>
+  </si>
+  <si>
+    <t xml:space="preserve">peptide_seq</t>
+  </si>
+  <si>
+    <t xml:space="preserve">affinity</t>
+  </si>
   <si>
     <t xml:space="preserve">PDZ</t>
   </si>
@@ -236,7 +248,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -249,119 +261,133 @@
       <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="n">
-        <v>8</v>
+      <c r="D1" s="3" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>100</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>1000</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="C4" s="3" t="s">
         <v>10</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>1000</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="3" t="n">
-        <v>10</v>
+      <c r="C5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>100</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D7" s="3" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D8" s="3" t="n">
         <v>700</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="D8" s="1" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B9" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="B9" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D9" s="3" t="n">
+      <c r="C9" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D9" s="1" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10" s="3" t="n">
         <v>22</v>
       </c>
     </row>

</xml_diff>